<commit_message>
Add worked example to lab5 Excel, reproducible build script, and deck backlog from /check-deck
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lab5/lab5_instr.xlsx
+++ b/lab5/lab5_instr.xlsx
@@ -9,13 +9,15 @@
   <sheets>
     <sheet name="Lab 5 Key" sheetId="1" r:id="rId1"/>
     <sheet name="Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Worked Example" sheetId="3" r:id="rId3"/>
+    <sheet name="Worked Data" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="109">
   <si>
     <t>Lab 5: Instructions and Walkthrough (Excel version)</t>
   </si>
@@ -264,6 +266,84 @@
   </si>
   <si>
     <t>R: set.seed(seed = 133); sleep_hours &lt;- round(rnorm(n = 10, mean = 6.5, sd = 0.9), digits = 1)</t>
+  </si>
+  <si>
+    <t>Lab 5 worked example (Excel version): weekly study hours</t>
+  </si>
+  <si>
+    <t>Yellow cells are inputs; change them and every answer updates. Raw data are on the Worked Data sheet.</t>
+  </si>
+  <si>
+    <t>Inputs: 12 students, H0: mu = 9, H_A: mu != 9 (two-tailed)</t>
+  </si>
+  <si>
+    <t>National average hours studied per week</t>
+  </si>
+  <si>
+    <t>mu_0 &lt;- 9</t>
+  </si>
+  <si>
+    <t>1. By hand: mean, s, standard error, and t</t>
+  </si>
+  <si>
+    <t>Count of the 12 scores on the Worked Data sheet</t>
+  </si>
+  <si>
+    <t>n &lt;- length(x = study_hours)</t>
+  </si>
+  <si>
+    <t>m &lt;- mean(x = study_hours)</t>
+  </si>
+  <si>
+    <t>sum((study_hours - m)^2)</t>
+  </si>
+  <si>
+    <t>s = sqrt(SS / (n - 1))</t>
+  </si>
+  <si>
+    <t>s &lt;- sd(x = study_hours)</t>
+  </si>
+  <si>
+    <t>SE = 4.72 / sqrt(12) = 1.36</t>
+  </si>
+  <si>
+    <t>t = (12.67 - 9) / 1.36 = 2.69: the mean is about 2.69 standard errors ABOVE 9</t>
+  </si>
+  <si>
+    <t>2. Degrees of freedom and critical value</t>
+  </si>
+  <si>
+    <t>df = n - 1 = 12 - 1 = 11</t>
+  </si>
+  <si>
+    <t>3. p-value, confidence interval, and decision</t>
+  </si>
+  <si>
+    <t>t.test(x = study_hours, mu = 9, alternative = "two.sided", conf.level = 0.95)$conf.int</t>
+  </si>
+  <si>
+    <t>mean + critical t x SE. The interval does NOT contain 9.</t>
+  </si>
+  <si>
+    <t>|t| = 2.69 &gt; 2.201 and p = .021 &lt; .05, so we reject H0. Students study more than the national average.</t>
+  </si>
+  <si>
+    <t>abs(x = t) &gt; t_crit</t>
+  </si>
+  <si>
+    <t>4. Effect size and APA sentence</t>
+  </si>
+  <si>
+    <t>d = (12.67 - 9) / 4.72 = 0.78</t>
+  </si>
+  <si>
+    <t>About 0.2 is small, 0.5 is medium, and 0.8 is large; 0.78 is at the medium/large boundary (the lab slides call it large, d ~ 0.8).</t>
+  </si>
+  <si>
+    <t>Study hours</t>
+  </si>
+  <si>
+    <t>R: set.seed(seed = 348); study_hours &lt;- round(x = rnorm(n = 12, mean = 12, sd = 4), digits = 0)</t>
   </si>
 </sst>
 </file>
@@ -863,7 +943,7 @@
       </c>
       <c r="B17" s="7">
         <f>(B13-$B$6)/B16</f>
-        <v>-2.0918294146798995</v>
+        <v>-2.091829414679899</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>37</v>
@@ -930,7 +1010,7 @@
       </c>
       <c r="B23" s="7">
         <f>T.INV($B$7,B21)</f>
-        <v>-1.8331129326562372</v>
+        <v>-1.833112932656237</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>47</v>
@@ -967,7 +1047,7 @@
       </c>
       <c r="B27" s="7">
         <f>T.DIST.2T(ABS(B17),B21)</f>
-        <v>0.0659872483695323</v>
+        <v>0.06598724836953228</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>51</v>
@@ -1049,7 +1129,7 @@
       </c>
       <c r="B34" s="7">
         <f>T.DIST(B17,B21,TRUE)</f>
-        <v>0.0329936241847661</v>
+        <v>0.03299362418476614</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>64</v>
@@ -1287,4 +1367,532 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="46.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="62.7109375" customWidth="1"/>
+    <col min="4" max="4" width="66.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="6">
+        <v>0.95</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="7">
+        <f>COUNT('Worked Data'!$B$2:$B$13)</f>
+        <v>12.0</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="7">
+        <f>AVERAGE('Worked Data'!$B$2:$B$13)</f>
+        <v>12.66666666666667</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="7">
+        <f>DEVSQ('Worked Data'!$B$2:$B$13)</f>
+        <v>244.6666666666667</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="7">
+        <f>STDEV.S('Worked Data'!$B$2:$B$13)</f>
+        <v>4.716187468965185</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="7">
+        <f>B15/SQRT(B12)</f>
+        <v>1.361446052377895</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="7">
+        <f>(B13-$B$6)/B16</f>
+        <v>2.693214806611312</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="7">
+        <f>B12-1</f>
+        <v>11.0</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" s="7">
+        <f>T.INV.2T($B$7,B21)</f>
+        <v>2.200985160091639</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="7">
+        <f>T.DIST.2T(ABS(B17),B21)</f>
+        <v>0.02090870511668394</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="7">
+        <f>B13-T.INV.2T(1-$B$8,B21)*B16</f>
+        <v>9.670144109117576</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="7">
+        <f>B13+T.INV.2T(1-$B$8,B21)*B16</f>
+        <v>15.66318922421576</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="8" t="str">
+        <f>IF(ABS(B17)&gt;B22,"Reject H0","Fail to reject H0")</f>
+        <v>Reject H0</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" s="7">
+        <f>(B13-$B$6)/B15</f>
+        <v>0.7774641467912634</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B34" s="8" t="str">
+        <f>IF(ABS(B33)&lt;0.2,"negligible",IF(ABS(B33)&lt;0.5,"small",IF(ABS(B33)&lt;0.8,"medium","large")))</f>
+        <v>medium</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="32" customHeight="1">
+      <c r="A35" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" s="5" t="str">
+        <f>"Students studied more than the national average of "&amp;TEXT($B$6,"0")&amp;" hours, M = "&amp;TEXT(B13,"0.00")&amp;", SD = "&amp;TEXT(B15,"0.00")&amp;", t("&amp;B21&amp;") = "&amp;TEXT(B17,"0.00")&amp;", p = "&amp;TEXT(B26,"0.000")&amp;", d = "&amp;TEXT(B33,"0.00")&amp;"."</f>
+        <v>Students studied more than the national average of 9 hours, M = 12.67, SD = 4.72, t(11) = 2.69, p = .021, d = 0.78.</v>
+      </c>
+      <c r="C35" s="5"/>
+      <c r="D35" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="B35:D35"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>